<commit_message>
TMTT0036857&TMTT0036859 DND Sharing CF&FR test cases
</commit_message>
<xml_diff>
--- a/TestData/TMTT0036859_VerifyTheFunctionalityOfDNDEngagementSharingFeatureForCFLOBOpportunityAndEngagementOnLightningView.xlsx
+++ b/TestData/TMTT0036859_VerifyTheFunctionalityOfDNDEngagementSharingFeatureForCFLOBOpportunityAndEngagementOnLightningView.xlsx
@@ -1,25 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26924"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27029"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vkumar0427\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49349C98-3E70-4933-84D6-0C1A378F870C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11C138CD-62D3-4ABB-89DC-EF7D006FA58E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="548" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="548" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="User" sheetId="2" r:id="rId1"/>
-    <sheet name="AppName" sheetId="3" r:id="rId2"/>
-    <sheet name="ModuleName" sheetId="4" r:id="rId3"/>
-    <sheet name="AddOpportunity" sheetId="12" r:id="rId4"/>
-    <sheet name="InternalTeams" sheetId="18" r:id="rId5"/>
-    <sheet name="AddContact" sheetId="14" r:id="rId6"/>
-    <sheet name="SharingGroup" sheetId="17" r:id="rId7"/>
+    <sheet name="StandardUser" sheetId="2" r:id="rId1"/>
+    <sheet name="CAOUser" sheetId="19" r:id="rId2"/>
+    <sheet name="DNDApprover" sheetId="20" r:id="rId3"/>
+    <sheet name="AppName" sheetId="3" r:id="rId4"/>
+    <sheet name="ModuleName" sheetId="4" r:id="rId5"/>
+    <sheet name="AddOpportunity" sheetId="12" r:id="rId6"/>
+    <sheet name="InternalTeams" sheetId="18" r:id="rId7"/>
+    <sheet name="AddContact" sheetId="14" r:id="rId8"/>
+    <sheet name="SharingGroup" sheetId="17" r:id="rId9"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="89">
   <si>
     <t>James Craven</t>
   </si>
@@ -152,9 +154,6 @@
     <t>RecordType</t>
   </si>
   <si>
-    <t>FASJobType</t>
-  </si>
-  <si>
     <t>MarketCap</t>
   </si>
   <si>
@@ -303,6 +302,15 @@
   </si>
   <si>
     <t>Drew Koecher</t>
+  </si>
+  <si>
+    <t>Engagements</t>
+  </si>
+  <si>
+    <t>Indrajeet Singh</t>
+  </si>
+  <si>
+    <t>System Administrator</t>
   </si>
 </sst>
 </file>
@@ -636,7 +644,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17" bestFit="1" customWidth="1"/>
@@ -652,37 +660,15 @@
         <v>2</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B2" t="s">
         <v>3</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3" t="s">
-        <v>10</v>
-      </c>
-      <c r="C3" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>78</v>
-      </c>
-      <c r="B4" t="s">
-        <v>10</v>
-      </c>
-      <c r="C4" t="s">
-        <v>79</v>
       </c>
     </row>
   </sheetData>
@@ -691,6 +677,86 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{204DA895-5616-4092-9340-8DD85852997B}">
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="12.5546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" t="s">
+        <v>80</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4767743C-3404-461F-B12D-D05F4986F9CF}">
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="13.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.33203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>77</v>
+      </c>
+      <c r="B2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>87</v>
+      </c>
+      <c r="B3" t="s">
+        <v>88</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0293C6CF-D2AF-4FB5-B989-23A4E6860FD2}">
   <dimension ref="A1:A2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -713,9 +779,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6D296AE2-31EA-40C7-99FB-9B7E70535054}">
-  <dimension ref="A1:A2"/>
+  <dimension ref="A1:A3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.5546875" bestFit="1" customWidth="1"/>
@@ -731,13 +797,18 @@
         <v>7</v>
       </c>
     </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>86</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AFD13242-055E-41A8-80D8-6F50F1B57F7C}">
   <dimension ref="A1:AE2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -746,8 +817,11 @@
     <col min="3" max="3" width="26.44140625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="26.88671875" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="12.77734375" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="11" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="16" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="11" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="11.109375" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="14.21875" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="16.77734375" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="14.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:31" x14ac:dyDescent="0.3">
@@ -827,117 +901,117 @@
         <v>35</v>
       </c>
       <c r="Z1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="AA1" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="AA1" s="1" t="s">
+      <c r="AB1" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="AB1" s="1" t="s">
+      <c r="AC1" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="AC1" s="1" t="s">
+      <c r="AD1" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="AD1" s="1" t="s">
-        <v>40</v>
-      </c>
       <c r="AE1" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="2" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C2" t="s">
+        <v>69</v>
+      </c>
+      <c r="D2" t="s">
         <v>41</v>
       </c>
-      <c r="B2" t="s">
-        <v>41</v>
-      </c>
-      <c r="C2" s="1" t="s">
+      <c r="E2" t="s">
+        <v>42</v>
+      </c>
+      <c r="F2" t="s">
+        <v>43</v>
+      </c>
+      <c r="G2" t="s">
+        <v>43</v>
+      </c>
+      <c r="H2" t="s">
+        <v>44</v>
+      </c>
+      <c r="I2" t="s">
+        <v>43</v>
+      </c>
+      <c r="J2" t="s">
+        <v>43</v>
+      </c>
+      <c r="K2" t="s">
         <v>70</v>
       </c>
-      <c r="D2" t="s">
-        <v>42</v>
-      </c>
-      <c r="E2" t="s">
-        <v>43</v>
-      </c>
-      <c r="F2" t="s">
-        <v>44</v>
-      </c>
-      <c r="G2" t="s">
-        <v>44</v>
-      </c>
-      <c r="H2" t="s">
+      <c r="L2" t="s">
         <v>45</v>
       </c>
-      <c r="I2" t="s">
-        <v>44</v>
-      </c>
-      <c r="J2" t="s">
-        <v>44</v>
-      </c>
-      <c r="K2" t="s">
-        <v>71</v>
-      </c>
-      <c r="L2" t="s">
+      <c r="M2" t="s">
         <v>46</v>
       </c>
-      <c r="M2" t="s">
+      <c r="N2" t="s">
+        <v>73</v>
+      </c>
+      <c r="O2" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="N2" t="s">
-        <v>74</v>
-      </c>
-      <c r="O2" s="3" t="s">
+      <c r="P2" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q2" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="R2" t="s">
         <v>48</v>
       </c>
-      <c r="P2" s="3" t="s">
+      <c r="S2" t="s">
         <v>48</v>
       </c>
-      <c r="Q2" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="R2" t="s">
+      <c r="T2" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="S2" t="s">
-        <v>49</v>
-      </c>
-      <c r="T2" s="3" t="s">
+      <c r="U2" t="s">
         <v>50</v>
       </c>
-      <c r="U2" t="s">
+      <c r="V2" t="s">
         <v>51</v>
       </c>
-      <c r="V2" t="s">
+      <c r="W2" t="s">
         <v>52</v>
       </c>
-      <c r="W2" t="s">
+      <c r="X2" t="s">
         <v>53</v>
       </c>
-      <c r="X2" t="s">
+      <c r="Y2" t="s">
         <v>54</v>
       </c>
-      <c r="Y2" t="s">
+      <c r="Z2" t="s">
         <v>55</v>
       </c>
-      <c r="Z2" t="s">
-        <v>56</v>
-      </c>
       <c r="AA2" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="AB2" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="AC2" t="s">
         <v>0</v>
       </c>
       <c r="AD2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="AE2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
   </sheetData>
@@ -946,7 +1020,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FFD3AFCB-FF3D-4430-A7EF-EB1CDD64D866}">
   <dimension ref="A1:A6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -956,7 +1030,7 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.3">
@@ -966,22 +1040,22 @@
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
   </sheetData>
@@ -989,7 +1063,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2F2CDCD2-7F5E-40FD-BAB3-4BCEC31CD21E}">
   <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1006,54 +1080,54 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>59</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>60</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>8</v>
       </c>
       <c r="E1" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>63</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>64</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B2" t="s">
+        <v>64</v>
+      </c>
+      <c r="C2" t="s">
         <v>65</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>66</v>
-      </c>
-      <c r="D2" t="s">
-        <v>67</v>
       </c>
       <c r="E2" t="s">
         <v>11</v>
       </c>
       <c r="F2" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G2" t="s">
         <v>11</v>
       </c>
       <c r="H2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
   </sheetData>
@@ -1061,7 +1135,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C2F5355-6C7D-4D28-98E4-51F296DA7AFE}">
   <dimension ref="A1:B2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1072,7 +1146,7 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>8</v>
@@ -1080,10 +1154,10 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
   </sheetData>

</xml_diff>